<commit_message>
chore(data): regenerate call listening xlsx
</commit_message>
<xml_diff>
--- a/data/coaching-tool-sync-backup.xlsx
+++ b/data/coaching-tool-sync-backup.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-02-25T16:41:05.683Z</t>
+          <t>2026-02-25T16:52:51.325Z</t>
         </is>
       </c>
     </row>
@@ -463,7 +463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>smoke-test 2026-02-25 09:41:06</t>
+          <t>validation-smoke</t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>smoke-test</t>
+          <t>validation-check</t>
         </is>
       </c>
     </row>

</xml_diff>